<commit_message>
Fix data inconsistencies: NetSuite label, 2026 cash receipts, .DS_Store
- Consolidated_Trial_Balance_MANUAL.xlsx README: source system for the
  Software entity said "QuickBooks Online"; it is NetSuite.
- Advisory GL and BofA bank statement contained 9 client payments
  (18 GL lines, $183,493) received Jan-Feb 2026 for Nov/Dec 2025
  invoices. They sorted into January because dates are mm/dd text.
  Removed them from the FY2025 files and recomputed the dependent
  figures: Advisory trial balance tab (true and formula columns),
  the Advisory tab and stacked tab in the consolidation workbook, and
  subsequent bank running balances. Those invoices are now correctly
  open AR at 12/31/2025.
- Remove committed .DS_Store and add .gitignore.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LUQbossvjjDKmYwiJZ73hY
</commit_message>
<xml_diff>
--- a/data/01_Corporate_Holdco/Consolidated_Trial_Balance_MANUAL.xlsx
+++ b/data/01_Corporate_Holdco/Consolidated_Trial_Balance_MANUAL.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB - Corporate" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB - Northbridge Software, Inc" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB - Verve Supply Co." sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB - Northbridge Advisory Grou" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated (unreviewed)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Known Issues" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TB - Corporate" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TB - Northbridge Software, Inc" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TB - Verve Supply Co." sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TB - Northbridge Advisory Grou" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Consolidated (unreviewed)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Known Issues" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Built by Priya in Excel each month by re-typing balances off four different exports (QuickBooks Online, Xero, a spreadsheet, and this workbook itself). No consolidation software, no shared chart of accounts, no elimination entries. This is genuinely the entire close process for the group.</t>
+          <t>Built by Priya in Excel each month by re-typing balances off four different exports (NetSuite, Xero, a spreadsheet, and this workbook itself). No consolidation software, no shared chart of accounts, no elimination entries. This is genuinely the entire close process for the group.</t>
         </is>
       </c>
     </row>
@@ -1740,10 +1740,10 @@
         <v>3582109</v>
       </c>
       <c r="C3" t="n">
-        <v>2626605.87</v>
+        <v>2443112.87</v>
       </c>
       <c r="D3" t="n">
-        <v>955503.13</v>
+        <v>1138996.13</v>
       </c>
     </row>
     <row r="4">
@@ -1753,13 +1753,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2609954</v>
+        <v>2426461</v>
       </c>
       <c r="C4" t="n">
         <v>3890556.8</v>
       </c>
       <c r="D4" t="n">
-        <v>-1280602.8</v>
+        <v>-1464095.8</v>
       </c>
     </row>
     <row r="5">
@@ -3565,10 +3565,10 @@
         <v>3582109</v>
       </c>
       <c r="D73" t="n">
-        <v>2626605.87</v>
+        <v>2443112.87</v>
       </c>
       <c r="E73" t="n">
-        <v>955503.13</v>
+        <v>1138996.13</v>
       </c>
     </row>
     <row r="74">
@@ -3583,13 +3583,13 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2609954</v>
+        <v>2426461</v>
       </c>
       <c r="D74" t="n">
         <v>3890556.8</v>
       </c>
       <c r="E74" t="n">
-        <v>-1280602.8</v>
+        <v>-1464095.8</v>
       </c>
     </row>
     <row r="75">

</xml_diff>